<commit_message>
PUS8 function correction + a bug fix for sweep bias
change of wrong N_samples_per_step_arg_id in command_data.py

bug removed for macro bias subwindow crash and wrong display in GUI .
</commit_message>
<xml_diff>
--- a/Macro_Sweep_Bias.xlsx
+++ b/Macro_Sweep_Bias.xlsx
@@ -457,47 +457,45 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>nof_act_sw_last_power_off</t>
+          <t>nstep_total_steps</t>
         </is>
       </c>
-      <c r="B3" t="n">
-        <v>0</v>
-      </c>
+      <c r="B3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>nof_steps_sb_mode</t>
+          <t>full_total_steps</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0</v>
+        <v>255</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>nof_samples_per_step</t>
+          <t>nof_act_sw_last_power_off</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>59245</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>nof_skipped_samples</t>
+          <t>nof_steps_sb_mode</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0</v>
+        <v>154</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>nof_samples_per_point</t>
+          <t>nof_samples_per_step</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -507,7 +505,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>nof_points_per_step</t>
+          <t>nof_skipped_samples</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -517,19 +515,21 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>nstep_total_steps_raw</t>
+          <t>nof_samples_per_point</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
+      <c r="B9" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>full_total_steps_raw</t>
+          <t>nof_points_per_step</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>255</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -599,10 +599,10 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>54781</v>
+        <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>40637</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -610,10 +610,10 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>32575</v>
+        <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>60373</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -621,10 +621,10 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>65367</v>
+        <v>2</v>
       </c>
       <c r="C4" t="n">
-        <v>55907</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5">
@@ -632,10 +632,10 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>54651</v>
+        <v>3</v>
       </c>
       <c r="C5" t="n">
-        <v>60119</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6">
@@ -643,10 +643,10 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>32349</v>
+        <v>4</v>
       </c>
       <c r="C6" t="n">
-        <v>40791</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7">
@@ -654,10 +654,10 @@
         <v>5</v>
       </c>
       <c r="B7" t="n">
-        <v>61439</v>
+        <v>5</v>
       </c>
       <c r="C7" t="n">
-        <v>65415</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8">
@@ -665,10 +665,10 @@
         <v>6</v>
       </c>
       <c r="B8" t="n">
-        <v>40573</v>
+        <v>6</v>
       </c>
       <c r="C8" t="n">
-        <v>49127</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9">
@@ -676,10 +676,10 @@
         <v>7</v>
       </c>
       <c r="B9" t="n">
-        <v>47581</v>
+        <v>7</v>
       </c>
       <c r="C9" t="n">
-        <v>56983</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10">
@@ -687,10 +687,10 @@
         <v>8</v>
       </c>
       <c r="B10" t="n">
-        <v>32637</v>
+        <v>8</v>
       </c>
       <c r="C10" t="n">
-        <v>65471</v>
+        <v>8</v>
       </c>
     </row>
     <row r="11">
@@ -698,10 +698,10 @@
         <v>9</v>
       </c>
       <c r="B11" t="n">
-        <v>15807</v>
+        <v>9</v>
       </c>
       <c r="C11" t="n">
-        <v>32767</v>
+        <v>9</v>
       </c>
     </row>
     <row r="12">
@@ -709,10 +709,10 @@
         <v>10</v>
       </c>
       <c r="B12" t="n">
-        <v>65503</v>
+        <v>10</v>
       </c>
       <c r="C12" t="n">
-        <v>24563</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13">
@@ -720,10 +720,10 @@
         <v>11</v>
       </c>
       <c r="B13" t="n">
-        <v>45023</v>
+        <v>11</v>
       </c>
       <c r="C13" t="n">
-        <v>30172</v>
+        <v>11</v>
       </c>
     </row>
     <row r="14">
@@ -731,10 +731,10 @@
         <v>12</v>
       </c>
       <c r="B14" t="n">
-        <v>65500</v>
+        <v>12</v>
       </c>
       <c r="C14" t="n">
-        <v>65503</v>
+        <v>12</v>
       </c>
     </row>
     <row r="15">
@@ -742,10 +742,10 @@
         <v>13</v>
       </c>
       <c r="B15" t="n">
-        <v>62749</v>
+        <v>13</v>
       </c>
       <c r="C15" t="n">
-        <v>16148</v>
+        <v>13</v>
       </c>
     </row>
     <row r="16">
@@ -753,10 +753,10 @@
         <v>14</v>
       </c>
       <c r="B16" t="n">
-        <v>40396</v>
+        <v>14</v>
       </c>
       <c r="C16" t="n">
-        <v>24561</v>
+        <v>14</v>
       </c>
     </row>
     <row r="17">
@@ -764,10 +764,10 @@
         <v>15</v>
       </c>
       <c r="B17" t="n">
-        <v>48247</v>
+        <v>15</v>
       </c>
       <c r="C17" t="n">
-        <v>30047</v>
+        <v>15</v>
       </c>
     </row>
     <row r="18">
@@ -775,10 +775,10 @@
         <v>16</v>
       </c>
       <c r="B18" t="n">
-        <v>13789</v>
+        <v>16</v>
       </c>
       <c r="C18" t="n">
-        <v>65211</v>
+        <v>16</v>
       </c>
     </row>
     <row r="19">
@@ -786,10 +786,10 @@
         <v>17</v>
       </c>
       <c r="B19" t="n">
-        <v>65527</v>
+        <v>17</v>
       </c>
       <c r="C19" t="n">
-        <v>13775</v>
+        <v>17</v>
       </c>
     </row>
     <row r="20">
@@ -797,10 +797,10 @@
         <v>18</v>
       </c>
       <c r="B20" t="n">
-        <v>65535</v>
+        <v>18</v>
       </c>
       <c r="C20" t="n">
-        <v>65507</v>
+        <v>18</v>
       </c>
     </row>
     <row r="21">
@@ -808,10 +808,10 @@
         <v>19</v>
       </c>
       <c r="B21" t="n">
-        <v>46941</v>
+        <v>19</v>
       </c>
       <c r="C21" t="n">
-        <v>24277</v>
+        <v>19</v>
       </c>
     </row>
     <row r="22">
@@ -819,10 +819,10 @@
         <v>20</v>
       </c>
       <c r="B22" t="n">
-        <v>64893</v>
+        <v>20</v>
       </c>
       <c r="C22" t="n">
-        <v>65211</v>
+        <v>20</v>
       </c>
     </row>
     <row r="23">
@@ -830,10 +830,10 @@
         <v>21</v>
       </c>
       <c r="B23" t="n">
-        <v>32759</v>
+        <v>21</v>
       </c>
       <c r="C23" t="n">
-        <v>32749</v>
+        <v>21</v>
       </c>
     </row>
     <row r="24">
@@ -841,10 +841,10 @@
         <v>22</v>
       </c>
       <c r="B24" t="n">
-        <v>46207</v>
+        <v>22</v>
       </c>
       <c r="C24" t="n">
-        <v>48967</v>
+        <v>22</v>
       </c>
     </row>
     <row r="25">
@@ -852,10 +852,10 @@
         <v>23</v>
       </c>
       <c r="B25" t="n">
-        <v>63383</v>
+        <v>23</v>
       </c>
       <c r="C25" t="n">
-        <v>49087</v>
+        <v>23</v>
       </c>
     </row>
     <row r="26">
@@ -863,10 +863,10 @@
         <v>24</v>
       </c>
       <c r="B26" t="n">
-        <v>15195</v>
+        <v>24</v>
       </c>
       <c r="C26" t="n">
-        <v>47070</v>
+        <v>24</v>
       </c>
     </row>
     <row r="27">
@@ -874,10 +874,10 @@
         <v>25</v>
       </c>
       <c r="B27" t="n">
-        <v>16185</v>
+        <v>25</v>
       </c>
       <c r="C27" t="n">
-        <v>26596</v>
+        <v>25</v>
       </c>
     </row>
     <row r="28">
@@ -885,10 +885,10 @@
         <v>26</v>
       </c>
       <c r="B28" t="n">
-        <v>48852</v>
+        <v>26</v>
       </c>
       <c r="C28" t="n">
-        <v>65351</v>
+        <v>26</v>
       </c>
     </row>
     <row r="29">
@@ -896,10 +896,10 @@
         <v>27</v>
       </c>
       <c r="B29" t="n">
-        <v>48095</v>
+        <v>27</v>
       </c>
       <c r="C29" t="n">
-        <v>64660</v>
+        <v>27</v>
       </c>
     </row>
     <row r="30">
@@ -907,10 +907,10 @@
         <v>28</v>
       </c>
       <c r="B30" t="n">
-        <v>28510</v>
+        <v>28</v>
       </c>
       <c r="C30" t="n">
-        <v>54173</v>
+        <v>28</v>
       </c>
     </row>
     <row r="31">
@@ -918,10 +918,10 @@
         <v>29</v>
       </c>
       <c r="B31" t="n">
-        <v>32633</v>
+        <v>29</v>
       </c>
       <c r="C31" t="n">
-        <v>32253</v>
+        <v>29</v>
       </c>
     </row>
     <row r="32">
@@ -929,10 +929,10 @@
         <v>30</v>
       </c>
       <c r="B32" t="n">
-        <v>59135</v>
+        <v>30</v>
       </c>
       <c r="C32" t="n">
-        <v>65265</v>
+        <v>30</v>
       </c>
     </row>
     <row r="33">
@@ -940,10 +940,10 @@
         <v>31</v>
       </c>
       <c r="B33" t="n">
-        <v>34815</v>
+        <v>31</v>
       </c>
       <c r="C33" t="n">
-        <v>62879</v>
+        <v>31</v>
       </c>
     </row>
     <row r="34">
@@ -951,10 +951,10 @@
         <v>32</v>
       </c>
       <c r="B34" t="n">
-        <v>32605</v>
+        <v>32</v>
       </c>
       <c r="C34" t="n">
-        <v>64255</v>
+        <v>32</v>
       </c>
     </row>
     <row r="35">
@@ -962,10 +962,10 @@
         <v>33</v>
       </c>
       <c r="B35" t="n">
-        <v>65084</v>
+        <v>33</v>
       </c>
       <c r="C35" t="n">
-        <v>65526</v>
+        <v>33</v>
       </c>
     </row>
     <row r="36">
@@ -973,10 +973,10 @@
         <v>34</v>
       </c>
       <c r="B36" t="n">
-        <v>65510</v>
+        <v>34</v>
       </c>
       <c r="C36" t="n">
-        <v>49135</v>
+        <v>34</v>
       </c>
     </row>
     <row r="37">
@@ -984,10 +984,10 @@
         <v>35</v>
       </c>
       <c r="B37" t="n">
-        <v>65439</v>
+        <v>35</v>
       </c>
       <c r="C37" t="n">
-        <v>31786</v>
+        <v>35</v>
       </c>
     </row>
     <row r="38">
@@ -995,10 +995,10 @@
         <v>36</v>
       </c>
       <c r="B38" t="n">
-        <v>31060</v>
+        <v>36</v>
       </c>
       <c r="C38" t="n">
-        <v>65013</v>
+        <v>36</v>
       </c>
     </row>
     <row r="39">
@@ -1006,10 +1006,10 @@
         <v>37</v>
       </c>
       <c r="B39" t="n">
-        <v>40831</v>
+        <v>37</v>
       </c>
       <c r="C39" t="n">
-        <v>20393</v>
+        <v>37</v>
       </c>
     </row>
     <row r="40">
@@ -1017,10 +1017,10 @@
         <v>38</v>
       </c>
       <c r="B40" t="n">
-        <v>65502</v>
+        <v>38</v>
       </c>
       <c r="C40" t="n">
-        <v>46457</v>
+        <v>38</v>
       </c>
     </row>
     <row r="41">
@@ -1028,10 +1028,10 @@
         <v>39</v>
       </c>
       <c r="B41" t="n">
-        <v>55295</v>
+        <v>39</v>
       </c>
       <c r="C41" t="n">
-        <v>32154</v>
+        <v>39</v>
       </c>
     </row>
     <row r="42">
@@ -1039,10 +1039,10 @@
         <v>40</v>
       </c>
       <c r="B42" t="n">
-        <v>30540</v>
+        <v>40</v>
       </c>
       <c r="C42" t="n">
-        <v>53971</v>
+        <v>40</v>
       </c>
     </row>
     <row r="43">
@@ -1050,10 +1050,10 @@
         <v>41</v>
       </c>
       <c r="B43" t="n">
-        <v>30556</v>
+        <v>41</v>
       </c>
       <c r="C43" t="n">
-        <v>12055</v>
+        <v>41</v>
       </c>
     </row>
     <row r="44">
@@ -1061,10 +1061,10 @@
         <v>42</v>
       </c>
       <c r="B44" t="n">
-        <v>46805</v>
+        <v>42</v>
       </c>
       <c r="C44" t="n">
-        <v>49005</v>
+        <v>42</v>
       </c>
     </row>
     <row r="45">
@@ -1072,10 +1072,10 @@
         <v>43</v>
       </c>
       <c r="B45" t="n">
-        <v>48639</v>
+        <v>43</v>
       </c>
       <c r="C45" t="n">
-        <v>62343</v>
+        <v>43</v>
       </c>
     </row>
     <row r="46">
@@ -1083,10 +1083,10 @@
         <v>44</v>
       </c>
       <c r="B46" t="n">
-        <v>32349</v>
+        <v>44</v>
       </c>
       <c r="C46" t="n">
-        <v>65466</v>
+        <v>44</v>
       </c>
     </row>
     <row r="47">
@@ -1094,10 +1094,10 @@
         <v>45</v>
       </c>
       <c r="B47" t="n">
-        <v>15829</v>
+        <v>45</v>
       </c>
       <c r="C47" t="n">
-        <v>48581</v>
+        <v>45</v>
       </c>
     </row>
     <row r="48">
@@ -1105,10 +1105,10 @@
         <v>46</v>
       </c>
       <c r="B48" t="n">
-        <v>65228</v>
+        <v>46</v>
       </c>
       <c r="C48" t="n">
-        <v>46696</v>
+        <v>46</v>
       </c>
     </row>
     <row r="49">
@@ -1116,10 +1116,10 @@
         <v>47</v>
       </c>
       <c r="B49" t="n">
-        <v>45017</v>
+        <v>47</v>
       </c>
       <c r="C49" t="n">
-        <v>60767</v>
+        <v>47</v>
       </c>
     </row>
     <row r="50">
@@ -1127,10 +1127,10 @@
         <v>48</v>
       </c>
       <c r="B50" t="n">
-        <v>14302</v>
+        <v>48</v>
       </c>
       <c r="C50" t="n">
-        <v>54535</v>
+        <v>48</v>
       </c>
     </row>
     <row r="51">
@@ -1138,10 +1138,10 @@
         <v>49</v>
       </c>
       <c r="B51" t="n">
-        <v>63323</v>
+        <v>49</v>
       </c>
       <c r="C51" t="n">
-        <v>32103</v>
+        <v>49</v>
       </c>
     </row>
     <row r="52">
@@ -1149,10 +1149,10 @@
         <v>50</v>
       </c>
       <c r="B52" t="n">
-        <v>65399</v>
+        <v>50</v>
       </c>
       <c r="C52" t="n">
-        <v>38897</v>
+        <v>50</v>
       </c>
     </row>
     <row r="53">
@@ -1160,10 +1160,10 @@
         <v>51</v>
       </c>
       <c r="B53" t="n">
-        <v>65023</v>
+        <v>51</v>
       </c>
       <c r="C53" t="n">
-        <v>61078</v>
+        <v>51</v>
       </c>
     </row>
     <row r="54">
@@ -1171,10 +1171,10 @@
         <v>52</v>
       </c>
       <c r="B54" t="n">
-        <v>14335</v>
+        <v>52</v>
       </c>
       <c r="C54" t="n">
-        <v>48891</v>
+        <v>52</v>
       </c>
     </row>
     <row r="55">
@@ -1182,10 +1182,10 @@
         <v>53</v>
       </c>
       <c r="B55" t="n">
-        <v>65365</v>
+        <v>53</v>
       </c>
       <c r="C55" t="n">
-        <v>60913</v>
+        <v>53</v>
       </c>
     </row>
     <row r="56">
@@ -1193,10 +1193,10 @@
         <v>54</v>
       </c>
       <c r="B56" t="n">
-        <v>40951</v>
+        <v>54</v>
       </c>
       <c r="C56" t="n">
-        <v>57317</v>
+        <v>54</v>
       </c>
     </row>
     <row r="57">
@@ -1204,10 +1204,10 @@
         <v>55</v>
       </c>
       <c r="B57" t="n">
-        <v>44565</v>
+        <v>55</v>
       </c>
       <c r="C57" t="n">
-        <v>48775</v>
+        <v>55</v>
       </c>
     </row>
     <row r="58">
@@ -1215,10 +1215,10 @@
         <v>56</v>
       </c>
       <c r="B58" t="n">
-        <v>62845</v>
+        <v>56</v>
       </c>
       <c r="C58" t="n">
-        <v>64254</v>
+        <v>56</v>
       </c>
     </row>
     <row r="59">
@@ -1226,10 +1226,10 @@
         <v>57</v>
       </c>
       <c r="B59" t="n">
-        <v>64827</v>
+        <v>57</v>
       </c>
       <c r="C59" t="n">
-        <v>62927</v>
+        <v>57</v>
       </c>
     </row>
     <row r="60">
@@ -1237,10 +1237,10 @@
         <v>58</v>
       </c>
       <c r="B60" t="n">
-        <v>49039</v>
+        <v>58</v>
       </c>
       <c r="C60" t="n">
-        <v>57187</v>
+        <v>58</v>
       </c>
     </row>
     <row r="61">
@@ -1248,10 +1248,10 @@
         <v>59</v>
       </c>
       <c r="B61" t="n">
-        <v>40411</v>
+        <v>59</v>
       </c>
       <c r="C61" t="n">
-        <v>58629</v>
+        <v>59</v>
       </c>
     </row>
     <row r="62">
@@ -1259,10 +1259,10 @@
         <v>60</v>
       </c>
       <c r="B62" t="n">
-        <v>30050</v>
+        <v>60</v>
       </c>
       <c r="C62" t="n">
-        <v>61119</v>
+        <v>60</v>
       </c>
     </row>
     <row r="63">
@@ -1270,10 +1270,10 @@
         <v>61</v>
       </c>
       <c r="B63" t="n">
-        <v>32209</v>
+        <v>61</v>
       </c>
       <c r="C63" t="n">
-        <v>7501</v>
+        <v>61</v>
       </c>
     </row>
     <row r="64">
@@ -1281,10 +1281,10 @@
         <v>62</v>
       </c>
       <c r="B64" t="n">
-        <v>64093</v>
+        <v>62</v>
       </c>
       <c r="C64" t="n">
-        <v>44855</v>
+        <v>62</v>
       </c>
     </row>
     <row r="65">
@@ -1292,10 +1292,10 @@
         <v>63</v>
       </c>
       <c r="B65" t="n">
-        <v>47103</v>
+        <v>63</v>
       </c>
       <c r="C65" t="n">
-        <v>65311</v>
+        <v>63</v>
       </c>
     </row>
     <row r="66">
@@ -1303,10 +1303,10 @@
         <v>64</v>
       </c>
       <c r="B66" t="n">
-        <v>24921</v>
+        <v>64</v>
       </c>
       <c r="C66" t="n">
-        <v>63229</v>
+        <v>64</v>
       </c>
     </row>
     <row r="67">
@@ -1314,10 +1314,10 @@
         <v>65</v>
       </c>
       <c r="B67" t="n">
-        <v>32639</v>
+        <v>65</v>
       </c>
       <c r="C67" t="n">
-        <v>32650</v>
+        <v>65</v>
       </c>
     </row>
     <row r="68">
@@ -1325,10 +1325,10 @@
         <v>66</v>
       </c>
       <c r="B68" t="n">
-        <v>40670</v>
+        <v>66</v>
       </c>
       <c r="C68" t="n">
-        <v>65507</v>
+        <v>66</v>
       </c>
     </row>
     <row r="69">
@@ -1336,10 +1336,10 @@
         <v>67</v>
       </c>
       <c r="B69" t="n">
-        <v>40495</v>
+        <v>67</v>
       </c>
       <c r="C69" t="n">
-        <v>31759</v>
+        <v>67</v>
       </c>
     </row>
     <row r="70">
@@ -1347,10 +1347,10 @@
         <v>68</v>
       </c>
       <c r="B70" t="n">
-        <v>14934</v>
+        <v>68</v>
       </c>
       <c r="C70" t="n">
-        <v>63484</v>
+        <v>68</v>
       </c>
     </row>
     <row r="71">
@@ -1358,10 +1358,10 @@
         <v>69</v>
       </c>
       <c r="B71" t="n">
-        <v>12287</v>
+        <v>69</v>
       </c>
       <c r="C71" t="n">
-        <v>13703</v>
+        <v>69</v>
       </c>
     </row>
     <row r="72">
@@ -1369,10 +1369,10 @@
         <v>70</v>
       </c>
       <c r="B72" t="n">
-        <v>48861</v>
+        <v>70</v>
       </c>
       <c r="C72" t="n">
-        <v>45305</v>
+        <v>70</v>
       </c>
     </row>
     <row r="73">
@@ -1380,10 +1380,10 @@
         <v>71</v>
       </c>
       <c r="B73" t="n">
-        <v>63229</v>
+        <v>71</v>
       </c>
       <c r="C73" t="n">
-        <v>64671</v>
+        <v>71</v>
       </c>
     </row>
     <row r="74">
@@ -1391,10 +1391,10 @@
         <v>72</v>
       </c>
       <c r="B74" t="n">
-        <v>32735</v>
+        <v>72</v>
       </c>
       <c r="C74" t="n">
-        <v>65215</v>
+        <v>72</v>
       </c>
     </row>
     <row r="75">
@@ -1402,10 +1402,10 @@
         <v>73</v>
       </c>
       <c r="B75" t="n">
-        <v>30623</v>
+        <v>73</v>
       </c>
       <c r="C75" t="n">
-        <v>48588</v>
+        <v>73</v>
       </c>
     </row>
     <row r="76">
@@ -1413,10 +1413,10 @@
         <v>74</v>
       </c>
       <c r="B76" t="n">
-        <v>63223</v>
+        <v>74</v>
       </c>
       <c r="C76" t="n">
-        <v>65411</v>
+        <v>74</v>
       </c>
     </row>
     <row r="77">
@@ -1424,10 +1424,10 @@
         <v>75</v>
       </c>
       <c r="B77" t="n">
-        <v>40303</v>
+        <v>75</v>
       </c>
       <c r="C77" t="n">
-        <v>48223</v>
+        <v>75</v>
       </c>
     </row>
     <row r="78">
@@ -1435,10 +1435,10 @@
         <v>76</v>
       </c>
       <c r="B78" t="n">
-        <v>32221</v>
+        <v>76</v>
       </c>
       <c r="C78" t="n">
-        <v>65499</v>
+        <v>76</v>
       </c>
     </row>
     <row r="79">
@@ -1446,10 +1446,10 @@
         <v>77</v>
       </c>
       <c r="B79" t="n">
-        <v>32059</v>
+        <v>77</v>
       </c>
       <c r="C79" t="n">
-        <v>65503</v>
+        <v>77</v>
       </c>
     </row>
     <row r="80">
@@ -1457,10 +1457,10 @@
         <v>78</v>
       </c>
       <c r="B80" t="n">
-        <v>40183</v>
+        <v>78</v>
       </c>
       <c r="C80" t="n">
-        <v>63397</v>
+        <v>78</v>
       </c>
     </row>
     <row r="81">
@@ -1468,10 +1468,10 @@
         <v>79</v>
       </c>
       <c r="B81" t="n">
-        <v>44255</v>
+        <v>79</v>
       </c>
       <c r="C81" t="n">
-        <v>30231</v>
+        <v>79</v>
       </c>
     </row>
     <row r="82">
@@ -1479,10 +1479,10 @@
         <v>80</v>
       </c>
       <c r="B82" t="n">
-        <v>29468</v>
+        <v>80</v>
       </c>
       <c r="C82" t="n">
-        <v>47871</v>
+        <v>80</v>
       </c>
     </row>
     <row r="83">
@@ -1490,10 +1490,10 @@
         <v>81</v>
       </c>
       <c r="B83" t="n">
-        <v>46591</v>
+        <v>81</v>
       </c>
       <c r="C83" t="n">
-        <v>64367</v>
+        <v>81</v>
       </c>
     </row>
     <row r="84">
@@ -1501,10 +1501,10 @@
         <v>82</v>
       </c>
       <c r="B84" t="n">
-        <v>48895</v>
+        <v>82</v>
       </c>
       <c r="C84" t="n">
-        <v>65321</v>
+        <v>82</v>
       </c>
     </row>
     <row r="85">
@@ -1512,10 +1512,10 @@
         <v>83</v>
       </c>
       <c r="B85" t="n">
-        <v>40317</v>
+        <v>83</v>
       </c>
       <c r="C85" t="n">
-        <v>64966</v>
+        <v>83</v>
       </c>
     </row>
     <row r="86">
@@ -1523,10 +1523,10 @@
         <v>84</v>
       </c>
       <c r="B86" t="n">
-        <v>30047</v>
+        <v>84</v>
       </c>
       <c r="C86" t="n">
-        <v>65247</v>
+        <v>84</v>
       </c>
     </row>
     <row r="87">
@@ -1534,10 +1534,10 @@
         <v>85</v>
       </c>
       <c r="B87" t="n">
-        <v>49049</v>
+        <v>85</v>
       </c>
       <c r="C87" t="n">
-        <v>55501</v>
+        <v>85</v>
       </c>
     </row>
     <row r="88">
@@ -1545,10 +1545,10 @@
         <v>86</v>
       </c>
       <c r="B88" t="n">
-        <v>65367</v>
+        <v>86</v>
       </c>
       <c r="C88" t="n">
-        <v>49083</v>
+        <v>86</v>
       </c>
     </row>
     <row r="89">
@@ -1556,10 +1556,10 @@
         <v>87</v>
       </c>
       <c r="B89" t="n">
-        <v>46941</v>
+        <v>87</v>
       </c>
       <c r="C89" t="n">
-        <v>11799</v>
+        <v>87</v>
       </c>
     </row>
     <row r="90">
@@ -1567,10 +1567,10 @@
         <v>88</v>
       </c>
       <c r="B90" t="n">
-        <v>32095</v>
+        <v>88</v>
       </c>
       <c r="C90" t="n">
-        <v>46297</v>
+        <v>88</v>
       </c>
     </row>
     <row r="91">
@@ -1578,10 +1578,10 @@
         <v>89</v>
       </c>
       <c r="B91" t="n">
-        <v>49051</v>
+        <v>89</v>
       </c>
       <c r="C91" t="n">
-        <v>30429</v>
+        <v>89</v>
       </c>
     </row>
     <row r="92">
@@ -1589,10 +1589,10 @@
         <v>90</v>
       </c>
       <c r="B92" t="n">
-        <v>41111</v>
+        <v>90</v>
       </c>
       <c r="C92" t="n">
-        <v>40945</v>
+        <v>90</v>
       </c>
     </row>
     <row r="93">
@@ -1600,10 +1600,10 @@
         <v>91</v>
       </c>
       <c r="B93" t="n">
-        <v>48509</v>
+        <v>91</v>
       </c>
       <c r="C93" t="n">
-        <v>60823</v>
+        <v>91</v>
       </c>
     </row>
     <row r="94">
@@ -1611,10 +1611,10 @@
         <v>92</v>
       </c>
       <c r="B94" t="n">
-        <v>64990</v>
+        <v>92</v>
       </c>
       <c r="C94" t="n">
-        <v>65501</v>
+        <v>92</v>
       </c>
     </row>
     <row r="95">
@@ -1622,10 +1622,10 @@
         <v>93</v>
       </c>
       <c r="B95" t="n">
-        <v>31615</v>
+        <v>93</v>
       </c>
       <c r="C95" t="n">
-        <v>32221</v>
+        <v>93</v>
       </c>
     </row>
     <row r="96">
@@ -1633,10 +1633,10 @@
         <v>94</v>
       </c>
       <c r="B96" t="n">
-        <v>65495</v>
+        <v>94</v>
       </c>
       <c r="C96" t="n">
-        <v>10218</v>
+        <v>94</v>
       </c>
     </row>
     <row r="97">
@@ -1644,10 +1644,10 @@
         <v>95</v>
       </c>
       <c r="B97" t="n">
-        <v>16381</v>
+        <v>95</v>
       </c>
       <c r="C97" t="n">
-        <v>20879</v>
+        <v>95</v>
       </c>
     </row>
     <row r="98">
@@ -1655,10 +1655,10 @@
         <v>96</v>
       </c>
       <c r="B98" t="n">
-        <v>32106</v>
+        <v>96</v>
       </c>
       <c r="C98" t="n">
-        <v>48477</v>
+        <v>96</v>
       </c>
     </row>
     <row r="99">
@@ -1666,10 +1666,10 @@
         <v>97</v>
       </c>
       <c r="B99" t="n">
-        <v>14253</v>
+        <v>97</v>
       </c>
       <c r="C99" t="n">
-        <v>56679</v>
+        <v>97</v>
       </c>
     </row>
     <row r="100">
@@ -1677,10 +1677,10 @@
         <v>98</v>
       </c>
       <c r="B100" t="n">
-        <v>47860</v>
+        <v>98</v>
       </c>
       <c r="C100" t="n">
-        <v>65472</v>
+        <v>98</v>
       </c>
     </row>
     <row r="101">
@@ -1688,10 +1688,10 @@
         <v>99</v>
       </c>
       <c r="B101" t="n">
-        <v>50638</v>
+        <v>99</v>
       </c>
       <c r="C101" t="n">
-        <v>57311</v>
+        <v>99</v>
       </c>
     </row>
     <row r="102">
@@ -1699,10 +1699,10 @@
         <v>100</v>
       </c>
       <c r="B102" t="n">
-        <v>62813</v>
+        <v>100</v>
       </c>
       <c r="C102" t="n">
-        <v>64425</v>
+        <v>100</v>
       </c>
     </row>
     <row r="103">
@@ -1710,10 +1710,10 @@
         <v>101</v>
       </c>
       <c r="B103" t="n">
-        <v>63358</v>
+        <v>101</v>
       </c>
       <c r="C103" t="n">
-        <v>28636</v>
+        <v>101</v>
       </c>
     </row>
     <row r="104">
@@ -1721,10 +1721,10 @@
         <v>102</v>
       </c>
       <c r="B104" t="n">
-        <v>65503</v>
+        <v>102</v>
       </c>
       <c r="C104" t="n">
-        <v>55091</v>
+        <v>102</v>
       </c>
     </row>
     <row r="105">
@@ -1732,10 +1732,10 @@
         <v>103</v>
       </c>
       <c r="B105" t="n">
-        <v>65375</v>
+        <v>103</v>
       </c>
       <c r="C105" t="n">
-        <v>65306</v>
+        <v>103</v>
       </c>
     </row>
     <row r="106">
@@ -1743,10 +1743,10 @@
         <v>104</v>
       </c>
       <c r="B106" t="n">
-        <v>30047</v>
+        <v>104</v>
       </c>
       <c r="C106" t="n">
-        <v>65531</v>
+        <v>104</v>
       </c>
     </row>
     <row r="107">
@@ -1754,10 +1754,10 @@
         <v>105</v>
       </c>
       <c r="B107" t="n">
-        <v>60917</v>
+        <v>105</v>
       </c>
       <c r="C107" t="n">
-        <v>36318</v>
+        <v>105</v>
       </c>
     </row>
     <row r="108">
@@ -1765,10 +1765,10 @@
         <v>106</v>
       </c>
       <c r="B108" t="n">
-        <v>57115</v>
+        <v>106</v>
       </c>
       <c r="C108" t="n">
-        <v>64482</v>
+        <v>106</v>
       </c>
     </row>
     <row r="109">
@@ -1776,10 +1776,10 @@
         <v>107</v>
       </c>
       <c r="B109" t="n">
-        <v>49143</v>
+        <v>107</v>
       </c>
       <c r="C109" t="n">
-        <v>29151</v>
+        <v>107</v>
       </c>
     </row>
     <row r="110">
@@ -1787,10 +1787,10 @@
         <v>108</v>
       </c>
       <c r="B110" t="n">
-        <v>63359</v>
+        <v>108</v>
       </c>
       <c r="C110" t="n">
-        <v>65211</v>
+        <v>108</v>
       </c>
     </row>
     <row r="111">
@@ -1798,10 +1798,10 @@
         <v>109</v>
       </c>
       <c r="B111" t="n">
-        <v>48635</v>
+        <v>109</v>
       </c>
       <c r="C111" t="n">
-        <v>58860</v>
+        <v>109</v>
       </c>
     </row>
     <row r="112">
@@ -1809,10 +1809,10 @@
         <v>110</v>
       </c>
       <c r="B112" t="n">
-        <v>65375</v>
+        <v>110</v>
       </c>
       <c r="C112" t="n">
-        <v>65535</v>
+        <v>110</v>
       </c>
     </row>
     <row r="113">
@@ -1820,10 +1820,10 @@
         <v>111</v>
       </c>
       <c r="B113" t="n">
-        <v>49117</v>
+        <v>111</v>
       </c>
       <c r="C113" t="n">
-        <v>64599</v>
+        <v>111</v>
       </c>
     </row>
     <row r="114">
@@ -1831,10 +1831,10 @@
         <v>112</v>
       </c>
       <c r="B114" t="n">
-        <v>32601</v>
+        <v>112</v>
       </c>
       <c r="C114" t="n">
-        <v>65215</v>
+        <v>112</v>
       </c>
     </row>
     <row r="115">
@@ -1842,10 +1842,10 @@
         <v>113</v>
       </c>
       <c r="B115" t="n">
-        <v>31767</v>
+        <v>113</v>
       </c>
       <c r="C115" t="n">
-        <v>24469</v>
+        <v>113</v>
       </c>
     </row>
     <row r="116">
@@ -1853,10 +1853,10 @@
         <v>114</v>
       </c>
       <c r="B116" t="n">
-        <v>49118</v>
+        <v>114</v>
       </c>
       <c r="C116" t="n">
-        <v>65195</v>
+        <v>114</v>
       </c>
     </row>
     <row r="117">
@@ -1864,10 +1864,10 @@
         <v>115</v>
       </c>
       <c r="B117" t="n">
-        <v>16381</v>
+        <v>115</v>
       </c>
       <c r="C117" t="n">
-        <v>65247</v>
+        <v>115</v>
       </c>
     </row>
     <row r="118">
@@ -1875,10 +1875,10 @@
         <v>116</v>
       </c>
       <c r="B118" t="n">
-        <v>32092</v>
+        <v>116</v>
       </c>
       <c r="C118" t="n">
-        <v>57236</v>
+        <v>116</v>
       </c>
     </row>
     <row r="119">
@@ -1886,10 +1886,10 @@
         <v>117</v>
       </c>
       <c r="B119" t="n">
-        <v>32189</v>
+        <v>117</v>
       </c>
       <c r="C119" t="n">
-        <v>14310</v>
+        <v>117</v>
       </c>
     </row>
     <row r="120">
@@ -1897,10 +1897,10 @@
         <v>118</v>
       </c>
       <c r="B120" t="n">
-        <v>40863</v>
+        <v>118</v>
       </c>
       <c r="C120" t="n">
-        <v>48099</v>
+        <v>118</v>
       </c>
     </row>
     <row r="121">
@@ -1908,10 +1908,10 @@
         <v>119</v>
       </c>
       <c r="B121" t="n">
-        <v>44796</v>
+        <v>119</v>
       </c>
       <c r="C121" t="n">
-        <v>32471</v>
+        <v>119</v>
       </c>
     </row>
     <row r="122">
@@ -1919,10 +1919,10 @@
         <v>120</v>
       </c>
       <c r="B122" t="n">
-        <v>31614</v>
+        <v>120</v>
       </c>
       <c r="C122" t="n">
-        <v>63289</v>
+        <v>120</v>
       </c>
     </row>
     <row r="123">
@@ -1930,10 +1930,10 @@
         <v>121</v>
       </c>
       <c r="B123" t="n">
-        <v>30587</v>
+        <v>121</v>
       </c>
       <c r="C123" t="n">
-        <v>29148</v>
+        <v>121</v>
       </c>
     </row>
     <row r="124">
@@ -1941,10 +1941,10 @@
         <v>122</v>
       </c>
       <c r="B124" t="n">
-        <v>46935</v>
+        <v>122</v>
       </c>
       <c r="C124" t="n">
-        <v>48639</v>
+        <v>122</v>
       </c>
     </row>
     <row r="125">
@@ -1952,10 +1952,10 @@
         <v>123</v>
       </c>
       <c r="B125" t="n">
-        <v>58239</v>
+        <v>123</v>
       </c>
       <c r="C125" t="n">
-        <v>49039</v>
+        <v>123</v>
       </c>
     </row>
     <row r="126">
@@ -1963,10 +1963,10 @@
         <v>124</v>
       </c>
       <c r="B126" t="n">
-        <v>46415</v>
+        <v>124</v>
       </c>
       <c r="C126" t="n">
-        <v>63710</v>
+        <v>124</v>
       </c>
     </row>
     <row r="127">
@@ -1974,10 +1974,10 @@
         <v>125</v>
       </c>
       <c r="B127" t="n">
-        <v>28511</v>
+        <v>125</v>
       </c>
       <c r="C127" t="n">
-        <v>65204</v>
+        <v>125</v>
       </c>
     </row>
     <row r="128">
@@ -1985,10 +1985,10 @@
         <v>126</v>
       </c>
       <c r="B128" t="n">
-        <v>49079</v>
+        <v>126</v>
       </c>
       <c r="C128" t="n">
-        <v>65534</v>
+        <v>126</v>
       </c>
     </row>
     <row r="129">
@@ -1996,10 +1996,10 @@
         <v>127</v>
       </c>
       <c r="B129" t="n">
-        <v>46811</v>
+        <v>127</v>
       </c>
       <c r="C129" t="n">
-        <v>65205</v>
+        <v>127</v>
       </c>
     </row>
     <row r="130">
@@ -2007,10 +2007,10 @@
         <v>128</v>
       </c>
       <c r="B130" t="n">
-        <v>30559</v>
+        <v>128</v>
       </c>
       <c r="C130" t="n">
-        <v>48127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="131">
@@ -2018,10 +2018,10 @@
         <v>129</v>
       </c>
       <c r="B131" t="n">
-        <v>13500</v>
+        <v>129</v>
       </c>
       <c r="C131" t="n">
-        <v>48414</v>
+        <v>129</v>
       </c>
     </row>
     <row r="132">
@@ -2029,10 +2029,10 @@
         <v>130</v>
       </c>
       <c r="B132" t="n">
-        <v>46997</v>
+        <v>130</v>
       </c>
       <c r="C132" t="n">
-        <v>32611</v>
+        <v>130</v>
       </c>
     </row>
     <row r="133">
@@ -2040,10 +2040,10 @@
         <v>131</v>
       </c>
       <c r="B133" t="n">
-        <v>60669</v>
+        <v>131</v>
       </c>
       <c r="C133" t="n">
-        <v>61327</v>
+        <v>131</v>
       </c>
     </row>
     <row r="134">
@@ -2051,10 +2051,10 @@
         <v>132</v>
       </c>
       <c r="B134" t="n">
-        <v>28441</v>
+        <v>132</v>
       </c>
       <c r="C134" t="n">
-        <v>57081</v>
+        <v>132</v>
       </c>
     </row>
     <row r="135">
@@ -2062,10 +2062,10 @@
         <v>133</v>
       </c>
       <c r="B135" t="n">
-        <v>54127</v>
+        <v>133</v>
       </c>
       <c r="C135" t="n">
-        <v>32467</v>
+        <v>133</v>
       </c>
     </row>
     <row r="136">
@@ -2073,10 +2073,10 @@
         <v>134</v>
       </c>
       <c r="B136" t="n">
-        <v>15335</v>
+        <v>134</v>
       </c>
       <c r="C136" t="n">
-        <v>47469</v>
+        <v>134</v>
       </c>
     </row>
     <row r="137">
@@ -2084,10 +2084,10 @@
         <v>135</v>
       </c>
       <c r="B137" t="n">
-        <v>30159</v>
+        <v>135</v>
       </c>
       <c r="C137" t="n">
-        <v>11597</v>
+        <v>135</v>
       </c>
     </row>
     <row r="138">
@@ -2095,10 +2095,10 @@
         <v>136</v>
       </c>
       <c r="B138" t="n">
-        <v>32606</v>
+        <v>136</v>
       </c>
       <c r="C138" t="n">
-        <v>65187</v>
+        <v>136</v>
       </c>
     </row>
     <row r="139">
@@ -2106,10 +2106,10 @@
         <v>137</v>
       </c>
       <c r="B139" t="n">
-        <v>64949</v>
+        <v>137</v>
       </c>
       <c r="C139" t="n">
-        <v>24050</v>
+        <v>137</v>
       </c>
     </row>
     <row r="140">
@@ -2117,10 +2117,10 @@
         <v>138</v>
       </c>
       <c r="B140" t="n">
-        <v>65239</v>
+        <v>138</v>
       </c>
       <c r="C140" t="n">
-        <v>65519</v>
+        <v>138</v>
       </c>
     </row>
     <row r="141">
@@ -2128,10 +2128,10 @@
         <v>139</v>
       </c>
       <c r="B141" t="n">
-        <v>40062</v>
+        <v>139</v>
       </c>
       <c r="C141" t="n">
-        <v>22999</v>
+        <v>139</v>
       </c>
     </row>
     <row r="142">
@@ -2139,10 +2139,10 @@
         <v>140</v>
       </c>
       <c r="B142" t="n">
-        <v>25956</v>
+        <v>140</v>
       </c>
       <c r="C142" t="n">
-        <v>63700</v>
+        <v>140</v>
       </c>
     </row>
     <row r="143">
@@ -2150,10 +2150,10 @@
         <v>141</v>
       </c>
       <c r="B143" t="n">
-        <v>6965</v>
+        <v>141</v>
       </c>
       <c r="C143" t="n">
-        <v>65420</v>
+        <v>141</v>
       </c>
     </row>
     <row r="144">
@@ -2161,10 +2161,10 @@
         <v>142</v>
       </c>
       <c r="B144" t="n">
-        <v>48797</v>
+        <v>142</v>
       </c>
       <c r="C144" t="n">
-        <v>65467</v>
+        <v>142</v>
       </c>
     </row>
     <row r="145">
@@ -2172,10 +2172,10 @@
         <v>143</v>
       </c>
       <c r="B145" t="n">
-        <v>38397</v>
+        <v>143</v>
       </c>
       <c r="C145" t="n">
-        <v>55197</v>
+        <v>143</v>
       </c>
     </row>
     <row r="146">
@@ -2183,10 +2183,10 @@
         <v>144</v>
       </c>
       <c r="B146" t="n">
-        <v>32093</v>
+        <v>144</v>
       </c>
       <c r="C146" t="n">
-        <v>60389</v>
+        <v>144</v>
       </c>
     </row>
     <row r="147">
@@ -2194,10 +2194,10 @@
         <v>145</v>
       </c>
       <c r="B147" t="n">
-        <v>30639</v>
+        <v>145</v>
       </c>
       <c r="C147" t="n">
-        <v>64679</v>
+        <v>145</v>
       </c>
     </row>
     <row r="148">
@@ -2205,10 +2205,10 @@
         <v>146</v>
       </c>
       <c r="B148" t="n">
-        <v>49055</v>
+        <v>146</v>
       </c>
       <c r="C148" t="n">
-        <v>6920</v>
+        <v>146</v>
       </c>
     </row>
     <row r="149">
@@ -2216,10 +2216,10 @@
         <v>147</v>
       </c>
       <c r="B149" t="n">
-        <v>43501</v>
+        <v>147</v>
       </c>
       <c r="C149" t="n">
-        <v>63830</v>
+        <v>147</v>
       </c>
     </row>
     <row r="150">
@@ -2227,10 +2227,10 @@
         <v>148</v>
       </c>
       <c r="B150" t="n">
-        <v>30029</v>
+        <v>148</v>
       </c>
       <c r="C150" t="n">
-        <v>65203</v>
+        <v>148</v>
       </c>
     </row>
     <row r="151">
@@ -2238,10 +2238,10 @@
         <v>149</v>
       </c>
       <c r="B151" t="n">
-        <v>65535</v>
+        <v>149</v>
       </c>
       <c r="C151" t="n">
-        <v>47828</v>
+        <v>149</v>
       </c>
     </row>
     <row r="152">
@@ -2249,10 +2249,10 @@
         <v>150</v>
       </c>
       <c r="B152" t="n">
-        <v>38524</v>
+        <v>150</v>
       </c>
       <c r="C152" t="n">
-        <v>14837</v>
+        <v>150</v>
       </c>
     </row>
     <row r="153">
@@ -2260,10 +2260,10 @@
         <v>151</v>
       </c>
       <c r="B153" t="n">
-        <v>37311</v>
+        <v>151</v>
       </c>
       <c r="C153" t="n">
-        <v>30853</v>
+        <v>151</v>
       </c>
     </row>
     <row r="154">
@@ -2271,10 +2271,10 @@
         <v>152</v>
       </c>
       <c r="B154" t="n">
-        <v>32092</v>
+        <v>152</v>
       </c>
       <c r="C154" t="n">
-        <v>63197</v>
+        <v>152</v>
       </c>
     </row>
     <row r="155">
@@ -2282,10 +2282,10 @@
         <v>153</v>
       </c>
       <c r="B155" t="n">
-        <v>32701</v>
+        <v>153</v>
       </c>
       <c r="C155" t="n">
-        <v>48863</v>
+        <v>153</v>
       </c>
     </row>
     <row r="156">
@@ -2293,10 +2293,10 @@
         <v>154</v>
       </c>
       <c r="B156" t="n">
-        <v>61270</v>
+        <v>154</v>
       </c>
       <c r="C156" t="n">
-        <v>21949</v>
+        <v>154</v>
       </c>
     </row>
     <row r="157">
@@ -2304,10 +2304,10 @@
         <v>155</v>
       </c>
       <c r="B157" t="n">
-        <v>47998</v>
+        <v>155</v>
       </c>
       <c r="C157" t="n">
-        <v>42389</v>
+        <v>155</v>
       </c>
     </row>
     <row r="158">
@@ -2315,10 +2315,10 @@
         <v>156</v>
       </c>
       <c r="B158" t="n">
-        <v>30293</v>
+        <v>156</v>
       </c>
       <c r="C158" t="n">
-        <v>31575</v>
+        <v>156</v>
       </c>
     </row>
     <row r="159">
@@ -2326,10 +2326,10 @@
         <v>157</v>
       </c>
       <c r="B159" t="n">
-        <v>31921</v>
+        <v>157</v>
       </c>
       <c r="C159" t="n">
-        <v>65022</v>
+        <v>157</v>
       </c>
     </row>
     <row r="160">
@@ -2337,10 +2337,10 @@
         <v>158</v>
       </c>
       <c r="B160" t="n">
-        <v>16318</v>
+        <v>158</v>
       </c>
       <c r="C160" t="n">
-        <v>45039</v>
+        <v>158</v>
       </c>
     </row>
     <row r="161">
@@ -2348,10 +2348,10 @@
         <v>159</v>
       </c>
       <c r="B161" t="n">
-        <v>60543</v>
+        <v>159</v>
       </c>
       <c r="C161" t="n">
-        <v>45340</v>
+        <v>159</v>
       </c>
     </row>
     <row r="162">
@@ -2359,10 +2359,10 @@
         <v>160</v>
       </c>
       <c r="B162" t="n">
-        <v>30559</v>
+        <v>160</v>
       </c>
       <c r="C162" t="n">
-        <v>65527</v>
+        <v>160</v>
       </c>
     </row>
     <row r="163">
@@ -2370,10 +2370,10 @@
         <v>161</v>
       </c>
       <c r="B163" t="n">
-        <v>65023</v>
+        <v>161</v>
       </c>
       <c r="C163" t="n">
-        <v>64989</v>
+        <v>161</v>
       </c>
     </row>
     <row r="164">
@@ -2381,10 +2381,10 @@
         <v>162</v>
       </c>
       <c r="B164" t="n">
-        <v>57046</v>
+        <v>162</v>
       </c>
       <c r="C164" t="n">
-        <v>30315</v>
+        <v>162</v>
       </c>
     </row>
     <row r="165">
@@ -2392,10 +2392,10 @@
         <v>163</v>
       </c>
       <c r="B165" t="n">
-        <v>36351</v>
+        <v>163</v>
       </c>
       <c r="C165" t="n">
-        <v>28118</v>
+        <v>163</v>
       </c>
     </row>
     <row r="166">
@@ -2403,10 +2403,10 @@
         <v>164</v>
       </c>
       <c r="B166" t="n">
-        <v>14175</v>
+        <v>164</v>
       </c>
       <c r="C166" t="n">
-        <v>45787</v>
+        <v>164</v>
       </c>
     </row>
     <row r="167">
@@ -2414,10 +2414,10 @@
         <v>165</v>
       </c>
       <c r="B167" t="n">
-        <v>16247</v>
+        <v>165</v>
       </c>
       <c r="C167" t="n">
-        <v>49127</v>
+        <v>165</v>
       </c>
     </row>
     <row r="168">
@@ -2425,10 +2425,10 @@
         <v>166</v>
       </c>
       <c r="B168" t="n">
-        <v>65430</v>
+        <v>166</v>
       </c>
       <c r="C168" t="n">
-        <v>62306</v>
+        <v>166</v>
       </c>
     </row>
     <row r="169">
@@ -2436,10 +2436,10 @@
         <v>167</v>
       </c>
       <c r="B169" t="n">
-        <v>6524</v>
+        <v>167</v>
       </c>
       <c r="C169" t="n">
-        <v>64989</v>
+        <v>167</v>
       </c>
     </row>
     <row r="170">
@@ -2447,10 +2447,10 @@
         <v>168</v>
       </c>
       <c r="B170" t="n">
-        <v>32607</v>
+        <v>168</v>
       </c>
       <c r="C170" t="n">
-        <v>29407</v>
+        <v>168</v>
       </c>
     </row>
     <row r="171">
@@ -2458,10 +2458,10 @@
         <v>169</v>
       </c>
       <c r="B171" t="n">
-        <v>30711</v>
+        <v>169</v>
       </c>
       <c r="C171" t="n">
-        <v>13257</v>
+        <v>169</v>
       </c>
     </row>
     <row r="172">
@@ -2469,10 +2469,10 @@
         <v>170</v>
       </c>
       <c r="B172" t="n">
-        <v>32455</v>
+        <v>170</v>
       </c>
       <c r="C172" t="n">
-        <v>65442</v>
+        <v>170</v>
       </c>
     </row>
     <row r="173">
@@ -2480,10 +2480,10 @@
         <v>171</v>
       </c>
       <c r="B173" t="n">
-        <v>8159</v>
+        <v>171</v>
       </c>
       <c r="C173" t="n">
-        <v>64423</v>
+        <v>171</v>
       </c>
     </row>
     <row r="174">
@@ -2491,10 +2491,10 @@
         <v>172</v>
       </c>
       <c r="B174" t="n">
-        <v>46404</v>
+        <v>172</v>
       </c>
       <c r="C174" t="n">
-        <v>56523</v>
+        <v>172</v>
       </c>
     </row>
     <row r="175">
@@ -2502,10 +2502,10 @@
         <v>173</v>
       </c>
       <c r="B175" t="n">
-        <v>58503</v>
+        <v>173</v>
       </c>
       <c r="C175" t="n">
-        <v>16190</v>
+        <v>173</v>
       </c>
     </row>
     <row r="176">
@@ -2513,10 +2513,10 @@
         <v>174</v>
       </c>
       <c r="B176" t="n">
-        <v>48942</v>
+        <v>174</v>
       </c>
       <c r="C176" t="n">
-        <v>40933</v>
+        <v>174</v>
       </c>
     </row>
     <row r="177">
@@ -2524,10 +2524,10 @@
         <v>175</v>
       </c>
       <c r="B177" t="n">
-        <v>42963</v>
+        <v>175</v>
       </c>
       <c r="C177" t="n">
-        <v>62623</v>
+        <v>175</v>
       </c>
     </row>
     <row r="178">
@@ -2535,10 +2535,10 @@
         <v>176</v>
       </c>
       <c r="B178" t="n">
-        <v>32093</v>
+        <v>176</v>
       </c>
       <c r="C178" t="n">
-        <v>63487</v>
+        <v>176</v>
       </c>
     </row>
     <row r="179">
@@ -2546,10 +2546,10 @@
         <v>177</v>
       </c>
       <c r="B179" t="n">
-        <v>60797</v>
+        <v>177</v>
       </c>
       <c r="C179" t="n">
-        <v>65452</v>
+        <v>177</v>
       </c>
     </row>
     <row r="180">
@@ -2557,10 +2557,10 @@
         <v>178</v>
       </c>
       <c r="B180" t="n">
-        <v>48853</v>
+        <v>178</v>
       </c>
       <c r="C180" t="n">
-        <v>49141</v>
+        <v>178</v>
       </c>
     </row>
     <row r="181">
@@ -2568,10 +2568,10 @@
         <v>179</v>
       </c>
       <c r="B181" t="n">
-        <v>40831</v>
+        <v>179</v>
       </c>
       <c r="C181" t="n">
-        <v>44423</v>
+        <v>179</v>
       </c>
     </row>
     <row r="182">
@@ -2579,10 +2579,10 @@
         <v>180</v>
       </c>
       <c r="B182" t="n">
-        <v>29788</v>
+        <v>180</v>
       </c>
       <c r="C182" t="n">
-        <v>65535</v>
+        <v>180</v>
       </c>
     </row>
     <row r="183">
@@ -2590,10 +2590,10 @@
         <v>181</v>
       </c>
       <c r="B183" t="n">
-        <v>63903</v>
+        <v>181</v>
       </c>
       <c r="C183" t="n">
-        <v>15701</v>
+        <v>181</v>
       </c>
     </row>
     <row r="184">
@@ -2601,10 +2601,10 @@
         <v>182</v>
       </c>
       <c r="B184" t="n">
-        <v>46975</v>
+        <v>182</v>
       </c>
       <c r="C184" t="n">
-        <v>64495</v>
+        <v>182</v>
       </c>
     </row>
     <row r="185">
@@ -2612,10 +2612,10 @@
         <v>183</v>
       </c>
       <c r="B185" t="n">
-        <v>48639</v>
+        <v>183</v>
       </c>
       <c r="C185" t="n">
-        <v>63435</v>
+        <v>183</v>
       </c>
     </row>
     <row r="186">
@@ -2623,10 +2623,10 @@
         <v>184</v>
       </c>
       <c r="B186" t="n">
-        <v>62805</v>
+        <v>184</v>
       </c>
       <c r="C186" t="n">
-        <v>48863</v>
+        <v>184</v>
       </c>
     </row>
     <row r="187">
@@ -2634,10 +2634,10 @@
         <v>185</v>
       </c>
       <c r="B187" t="n">
-        <v>47037</v>
+        <v>185</v>
       </c>
       <c r="C187" t="n">
-        <v>49140</v>
+        <v>185</v>
       </c>
     </row>
     <row r="188">
@@ -2645,10 +2645,10 @@
         <v>186</v>
       </c>
       <c r="B188" t="n">
-        <v>49117</v>
+        <v>186</v>
       </c>
       <c r="C188" t="n">
-        <v>38847</v>
+        <v>186</v>
       </c>
     </row>
     <row r="189">
@@ -2656,10 +2656,10 @@
         <v>187</v>
       </c>
       <c r="B189" t="n">
-        <v>45007</v>
+        <v>187</v>
       </c>
       <c r="C189" t="n">
-        <v>60925</v>
+        <v>187</v>
       </c>
     </row>
     <row r="190">
@@ -2667,10 +2667,10 @@
         <v>188</v>
       </c>
       <c r="B190" t="n">
-        <v>65005</v>
+        <v>188</v>
       </c>
       <c r="C190" t="n">
-        <v>55547</v>
+        <v>188</v>
       </c>
     </row>
     <row r="191">
@@ -2678,10 +2678,10 @@
         <v>189</v>
       </c>
       <c r="B191" t="n">
-        <v>16127</v>
+        <v>189</v>
       </c>
       <c r="C191" t="n">
-        <v>45036</v>
+        <v>189</v>
       </c>
     </row>
     <row r="192">
@@ -2689,10 +2689,10 @@
         <v>190</v>
       </c>
       <c r="B192" t="n">
-        <v>38852</v>
+        <v>190</v>
       </c>
       <c r="C192" t="n">
-        <v>65251</v>
+        <v>190</v>
       </c>
     </row>
     <row r="193">
@@ -2700,10 +2700,10 @@
         <v>191</v>
       </c>
       <c r="B193" t="n">
-        <v>56062</v>
+        <v>191</v>
       </c>
       <c r="C193" t="n">
-        <v>54303</v>
+        <v>191</v>
       </c>
     </row>
     <row r="194">
@@ -2711,10 +2711,10 @@
         <v>192</v>
       </c>
       <c r="B194" t="n">
-        <v>30068</v>
+        <v>192</v>
       </c>
       <c r="C194" t="n">
-        <v>54079</v>
+        <v>192</v>
       </c>
     </row>
     <row r="195">
@@ -2722,10 +2722,10 @@
         <v>193</v>
       </c>
       <c r="B195" t="n">
-        <v>64799</v>
+        <v>193</v>
       </c>
       <c r="C195" t="n">
-        <v>32239</v>
+        <v>193</v>
       </c>
     </row>
     <row r="196">
@@ -2733,10 +2733,10 @@
         <v>194</v>
       </c>
       <c r="B196" t="n">
-        <v>49076</v>
+        <v>194</v>
       </c>
       <c r="C196" t="n">
-        <v>65511</v>
+        <v>194</v>
       </c>
     </row>
     <row r="197">
@@ -2744,10 +2744,10 @@
         <v>195</v>
       </c>
       <c r="B197" t="n">
-        <v>64511</v>
+        <v>195</v>
       </c>
       <c r="C197" t="n">
-        <v>44245</v>
+        <v>195</v>
       </c>
     </row>
     <row r="198">
@@ -2755,10 +2755,10 @@
         <v>196</v>
       </c>
       <c r="B198" t="n">
-        <v>30058</v>
+        <v>196</v>
       </c>
       <c r="C198" t="n">
-        <v>54015</v>
+        <v>196</v>
       </c>
     </row>
     <row r="199">
@@ -2766,10 +2766,10 @@
         <v>197</v>
       </c>
       <c r="B199" t="n">
-        <v>62262</v>
+        <v>197</v>
       </c>
       <c r="C199" t="n">
-        <v>15203</v>
+        <v>197</v>
       </c>
     </row>
     <row r="200">
@@ -2777,10 +2777,10 @@
         <v>198</v>
       </c>
       <c r="B200" t="n">
-        <v>48987</v>
+        <v>198</v>
       </c>
       <c r="C200" t="n">
-        <v>63843</v>
+        <v>198</v>
       </c>
     </row>
     <row r="201">
@@ -2788,10 +2788,10 @@
         <v>199</v>
       </c>
       <c r="B201" t="n">
-        <v>37823</v>
+        <v>199</v>
       </c>
       <c r="C201" t="n">
-        <v>64539</v>
+        <v>199</v>
       </c>
     </row>
     <row r="202">
@@ -2799,10 +2799,10 @@
         <v>200</v>
       </c>
       <c r="B202" t="n">
-        <v>32094</v>
+        <v>200</v>
       </c>
       <c r="C202" t="n">
-        <v>55033</v>
+        <v>200</v>
       </c>
     </row>
     <row r="203">
@@ -2810,10 +2810,10 @@
         <v>201</v>
       </c>
       <c r="B203" t="n">
-        <v>29999</v>
+        <v>201</v>
       </c>
       <c r="C203" t="n">
-        <v>32479</v>
+        <v>201</v>
       </c>
     </row>
     <row r="204">
@@ -2821,10 +2821,10 @@
         <v>202</v>
       </c>
       <c r="B204" t="n">
-        <v>65486</v>
+        <v>202</v>
       </c>
       <c r="C204" t="n">
-        <v>40811</v>
+        <v>202</v>
       </c>
     </row>
     <row r="205">
@@ -2832,10 +2832,10 @@
         <v>203</v>
       </c>
       <c r="B205" t="n">
-        <v>45407</v>
+        <v>203</v>
       </c>
       <c r="C205" t="n">
-        <v>26927</v>
+        <v>203</v>
       </c>
     </row>
     <row r="206">
@@ -2843,10 +2843,10 @@
         <v>204</v>
       </c>
       <c r="B206" t="n">
-        <v>32533</v>
+        <v>204</v>
       </c>
       <c r="C206" t="n">
-        <v>32503</v>
+        <v>204</v>
       </c>
     </row>
     <row r="207">
@@ -2854,10 +2854,10 @@
         <v>205</v>
       </c>
       <c r="B207" t="n">
-        <v>65329</v>
+        <v>205</v>
       </c>
       <c r="C207" t="n">
-        <v>15815</v>
+        <v>205</v>
       </c>
     </row>
     <row r="208">
@@ -2865,10 +2865,10 @@
         <v>206</v>
       </c>
       <c r="B208" t="n">
-        <v>46823</v>
+        <v>206</v>
       </c>
       <c r="C208" t="n">
-        <v>46970</v>
+        <v>206</v>
       </c>
     </row>
     <row r="209">
@@ -2876,10 +2876,10 @@
         <v>207</v>
       </c>
       <c r="B209" t="n">
-        <v>46251</v>
+        <v>207</v>
       </c>
       <c r="C209" t="n">
-        <v>62235</v>
+        <v>207</v>
       </c>
     </row>
     <row r="210">
@@ -2887,10 +2887,10 @@
         <v>208</v>
       </c>
       <c r="B210" t="n">
-        <v>30681</v>
+        <v>208</v>
       </c>
       <c r="C210" t="n">
-        <v>52441</v>
+        <v>208</v>
       </c>
     </row>
     <row r="211">
@@ -2898,10 +2898,10 @@
         <v>209</v>
       </c>
       <c r="B211" t="n">
-        <v>10239</v>
+        <v>209</v>
       </c>
       <c r="C211" t="n">
-        <v>48583</v>
+        <v>209</v>
       </c>
     </row>
     <row r="212">
@@ -2909,10 +2909,10 @@
         <v>210</v>
       </c>
       <c r="B212" t="n">
-        <v>61143</v>
+        <v>210</v>
       </c>
       <c r="C212" t="n">
-        <v>56610</v>
+        <v>210</v>
       </c>
     </row>
     <row r="213">
@@ -2920,10 +2920,10 @@
         <v>211</v>
       </c>
       <c r="B213" t="n">
-        <v>64972</v>
+        <v>211</v>
       </c>
       <c r="C213" t="n">
-        <v>65414</v>
+        <v>211</v>
       </c>
     </row>
     <row r="214">
@@ -2931,10 +2931,10 @@
         <v>212</v>
       </c>
       <c r="B214" t="n">
-        <v>54715</v>
+        <v>212</v>
       </c>
       <c r="C214" t="n">
-        <v>62606</v>
+        <v>212</v>
       </c>
     </row>
     <row r="215">
@@ -2942,10 +2942,10 @@
         <v>213</v>
       </c>
       <c r="B215" t="n">
-        <v>44671</v>
+        <v>213</v>
       </c>
       <c r="C215" t="n">
-        <v>63263</v>
+        <v>213</v>
       </c>
     </row>
     <row r="216">
@@ -2953,10 +2953,10 @@
         <v>214</v>
       </c>
       <c r="B216" t="n">
-        <v>53212</v>
+        <v>214</v>
       </c>
       <c r="C216" t="n">
-        <v>24363</v>
+        <v>214</v>
       </c>
     </row>
     <row r="217">
@@ -2964,10 +2964,10 @@
         <v>215</v>
       </c>
       <c r="B217" t="n">
-        <v>42359</v>
+        <v>215</v>
       </c>
       <c r="C217" t="n">
-        <v>11421</v>
+        <v>215</v>
       </c>
     </row>
     <row r="218">
@@ -2975,10 +2975,10 @@
         <v>216</v>
       </c>
       <c r="B218" t="n">
-        <v>32078</v>
+        <v>216</v>
       </c>
       <c r="C218" t="n">
-        <v>63455</v>
+        <v>216</v>
       </c>
     </row>
     <row r="219">
@@ -2986,10 +2986,10 @@
         <v>217</v>
       </c>
       <c r="B219" t="n">
-        <v>40319</v>
+        <v>217</v>
       </c>
       <c r="C219" t="n">
-        <v>32193</v>
+        <v>217</v>
       </c>
     </row>
     <row r="220">
@@ -2997,10 +2997,10 @@
         <v>218</v>
       </c>
       <c r="B220" t="n">
-        <v>49149</v>
+        <v>218</v>
       </c>
       <c r="C220" t="n">
-        <v>40943</v>
+        <v>218</v>
       </c>
     </row>
     <row r="221">
@@ -3008,10 +3008,10 @@
         <v>219</v>
       </c>
       <c r="B221" t="n">
-        <v>62847</v>
+        <v>219</v>
       </c>
       <c r="C221" t="n">
-        <v>63231</v>
+        <v>219</v>
       </c>
     </row>
     <row r="222">
@@ -3019,10 +3019,10 @@
         <v>220</v>
       </c>
       <c r="B222" t="n">
-        <v>32598</v>
+        <v>220</v>
       </c>
       <c r="C222" t="n">
-        <v>47327</v>
+        <v>220</v>
       </c>
     </row>
     <row r="223">
@@ -3030,10 +3030,10 @@
         <v>221</v>
       </c>
       <c r="B223" t="n">
-        <v>32189</v>
+        <v>221</v>
       </c>
       <c r="C223" t="n">
-        <v>15733</v>
+        <v>221</v>
       </c>
     </row>
     <row r="224">
@@ -3041,10 +3041,10 @@
         <v>222</v>
       </c>
       <c r="B224" t="n">
-        <v>65183</v>
+        <v>222</v>
       </c>
       <c r="C224" t="n">
-        <v>64319</v>
+        <v>222</v>
       </c>
     </row>
     <row r="225">
@@ -3052,10 +3052,10 @@
         <v>223</v>
       </c>
       <c r="B225" t="n">
-        <v>46975</v>
+        <v>223</v>
       </c>
       <c r="C225" t="n">
-        <v>57323</v>
+        <v>223</v>
       </c>
     </row>
     <row r="226">
@@ -3063,10 +3063,10 @@
         <v>224</v>
       </c>
       <c r="B226" t="n">
-        <v>29981</v>
+        <v>224</v>
       </c>
       <c r="C226" t="n">
-        <v>62843</v>
+        <v>224</v>
       </c>
     </row>
     <row r="227">
@@ -3074,10 +3074,10 @@
         <v>225</v>
       </c>
       <c r="B227" t="n">
-        <v>65515</v>
+        <v>225</v>
       </c>
       <c r="C227" t="n">
-        <v>49095</v>
+        <v>225</v>
       </c>
     </row>
     <row r="228">
@@ -3085,10 +3085,10 @@
         <v>226</v>
       </c>
       <c r="B228" t="n">
-        <v>65239</v>
+        <v>226</v>
       </c>
       <c r="C228" t="n">
-        <v>63462</v>
+        <v>226</v>
       </c>
     </row>
     <row r="229">
@@ -3096,10 +3096,10 @@
         <v>227</v>
       </c>
       <c r="B229" t="n">
-        <v>64759</v>
+        <v>227</v>
       </c>
       <c r="C229" t="n">
-        <v>42123</v>
+        <v>227</v>
       </c>
     </row>
     <row r="230">
@@ -3107,10 +3107,10 @@
         <v>228</v>
       </c>
       <c r="B230" t="n">
-        <v>46556</v>
+        <v>228</v>
       </c>
       <c r="C230" t="n">
-        <v>32379</v>
+        <v>228</v>
       </c>
     </row>
     <row r="231">
@@ -3118,10 +3118,10 @@
         <v>229</v>
       </c>
       <c r="B231" t="n">
-        <v>65495</v>
+        <v>229</v>
       </c>
       <c r="C231" t="n">
-        <v>4049</v>
+        <v>229</v>
       </c>
     </row>
     <row r="232">
@@ -3129,10 +3129,10 @@
         <v>230</v>
       </c>
       <c r="B232" t="n">
-        <v>40916</v>
+        <v>230</v>
       </c>
       <c r="C232" t="n">
-        <v>39909</v>
+        <v>230</v>
       </c>
     </row>
     <row r="233">
@@ -3140,10 +3140,10 @@
         <v>231</v>
       </c>
       <c r="B233" t="n">
-        <v>56809</v>
+        <v>231</v>
       </c>
       <c r="C233" t="n">
-        <v>64486</v>
+        <v>231</v>
       </c>
     </row>
     <row r="234">
@@ -3151,10 +3151,10 @@
         <v>232</v>
       </c>
       <c r="B234" t="n">
-        <v>29821</v>
+        <v>232</v>
       </c>
       <c r="C234" t="n">
-        <v>31613</v>
+        <v>232</v>
       </c>
     </row>
     <row r="235">
@@ -3162,10 +3162,10 @@
         <v>233</v>
       </c>
       <c r="B235" t="n">
-        <v>32633</v>
+        <v>233</v>
       </c>
       <c r="C235" t="n">
-        <v>28436</v>
+        <v>233</v>
       </c>
     </row>
     <row r="236">
@@ -3173,10 +3173,10 @@
         <v>234</v>
       </c>
       <c r="B236" t="n">
-        <v>38901</v>
+        <v>234</v>
       </c>
       <c r="C236" t="n">
-        <v>48098</v>
+        <v>234</v>
       </c>
     </row>
     <row r="237">
@@ -3184,10 +3184,10 @@
         <v>235</v>
       </c>
       <c r="B237" t="n">
-        <v>15215</v>
+        <v>235</v>
       </c>
       <c r="C237" t="n">
-        <v>63902</v>
+        <v>235</v>
       </c>
     </row>
     <row r="238">
@@ -3195,10 +3195,10 @@
         <v>236</v>
       </c>
       <c r="B238" t="n">
-        <v>63326</v>
+        <v>236</v>
       </c>
       <c r="C238" t="n">
-        <v>56231</v>
+        <v>236</v>
       </c>
     </row>
     <row r="239">
@@ -3206,10 +3206,10 @@
         <v>237</v>
       </c>
       <c r="B239" t="n">
-        <v>14239</v>
+        <v>237</v>
       </c>
       <c r="C239" t="n">
-        <v>15879</v>
+        <v>237</v>
       </c>
     </row>
     <row r="240">
@@ -3217,10 +3217,10 @@
         <v>238</v>
       </c>
       <c r="B240" t="n">
-        <v>48855</v>
+        <v>238</v>
       </c>
       <c r="C240" t="n">
-        <v>57067</v>
+        <v>238</v>
       </c>
     </row>
     <row r="241">
@@ -3228,10 +3228,10 @@
         <v>239</v>
       </c>
       <c r="B241" t="n">
-        <v>6652</v>
+        <v>239</v>
       </c>
       <c r="C241" t="n">
-        <v>46749</v>
+        <v>239</v>
       </c>
     </row>
     <row r="242">
@@ -3239,10 +3239,10 @@
         <v>240</v>
       </c>
       <c r="B242" t="n">
-        <v>29021</v>
+        <v>240</v>
       </c>
       <c r="C242" t="n">
-        <v>65527</v>
+        <v>240</v>
       </c>
     </row>
     <row r="243">
@@ -3250,10 +3250,10 @@
         <v>241</v>
       </c>
       <c r="B243" t="n">
-        <v>46847</v>
+        <v>241</v>
       </c>
       <c r="C243" t="n">
-        <v>60749</v>
+        <v>241</v>
       </c>
     </row>
     <row r="244">
@@ -3261,10 +3261,10 @@
         <v>242</v>
       </c>
       <c r="B244" t="n">
-        <v>48791</v>
+        <v>242</v>
       </c>
       <c r="C244" t="n">
-        <v>65487</v>
+        <v>242</v>
       </c>
     </row>
     <row r="245">
@@ -3272,10 +3272,10 @@
         <v>243</v>
       </c>
       <c r="B245" t="n">
-        <v>48631</v>
+        <v>243</v>
       </c>
       <c r="C245" t="n">
-        <v>49035</v>
+        <v>243</v>
       </c>
     </row>
     <row r="246">
@@ -3283,10 +3283,10 @@
         <v>244</v>
       </c>
       <c r="B246" t="n">
-        <v>30585</v>
+        <v>244</v>
       </c>
       <c r="C246" t="n">
-        <v>57064</v>
+        <v>244</v>
       </c>
     </row>
     <row r="247">
@@ -3294,10 +3294,10 @@
         <v>245</v>
       </c>
       <c r="B247" t="n">
-        <v>65471</v>
+        <v>245</v>
       </c>
       <c r="C247" t="n">
-        <v>15685</v>
+        <v>245</v>
       </c>
     </row>
     <row r="248">
@@ -3305,10 +3305,10 @@
         <v>246</v>
       </c>
       <c r="B248" t="n">
-        <v>40957</v>
+        <v>246</v>
       </c>
       <c r="C248" t="n">
-        <v>61434</v>
+        <v>246</v>
       </c>
     </row>
     <row r="249">
@@ -3316,10 +3316,10 @@
         <v>247</v>
       </c>
       <c r="B249" t="n">
-        <v>14125</v>
+        <v>247</v>
       </c>
       <c r="C249" t="n">
-        <v>21903</v>
+        <v>247</v>
       </c>
     </row>
     <row r="250">
@@ -3327,10 +3327,10 @@
         <v>248</v>
       </c>
       <c r="B250" t="n">
-        <v>15836</v>
+        <v>248</v>
       </c>
       <c r="C250" t="n">
-        <v>32479</v>
+        <v>248</v>
       </c>
     </row>
     <row r="251">
@@ -3338,10 +3338,10 @@
         <v>249</v>
       </c>
       <c r="B251" t="n">
-        <v>47003</v>
+        <v>249</v>
       </c>
       <c r="C251" t="n">
-        <v>32725</v>
+        <v>249</v>
       </c>
     </row>
     <row r="252">
@@ -3349,10 +3349,10 @@
         <v>250</v>
       </c>
       <c r="B252" t="n">
-        <v>55223</v>
+        <v>250</v>
       </c>
       <c r="C252" t="n">
-        <v>28623</v>
+        <v>250</v>
       </c>
     </row>
     <row r="253">
@@ -3360,10 +3360,10 @@
         <v>251</v>
       </c>
       <c r="B253" t="n">
-        <v>65535</v>
+        <v>251</v>
       </c>
       <c r="C253" t="n">
-        <v>30895</v>
+        <v>251</v>
       </c>
     </row>
     <row r="254">
@@ -3371,10 +3371,10 @@
         <v>252</v>
       </c>
       <c r="B254" t="n">
-        <v>30559</v>
+        <v>252</v>
       </c>
       <c r="C254" t="n">
-        <v>48895</v>
+        <v>252</v>
       </c>
     </row>
     <row r="255">
@@ -3382,10 +3382,10 @@
         <v>253</v>
       </c>
       <c r="B255" t="n">
-        <v>56893</v>
+        <v>253</v>
       </c>
       <c r="C255" t="n">
-        <v>64965</v>
+        <v>253</v>
       </c>
     </row>
     <row r="256">
@@ -3393,10 +3393,10 @@
         <v>254</v>
       </c>
       <c r="B256" t="n">
-        <v>49119</v>
+        <v>254</v>
       </c>
       <c r="C256" t="n">
-        <v>63471</v>
+        <v>254</v>
       </c>
     </row>
     <row r="257">
@@ -3404,10 +3404,10 @@
         <v>255</v>
       </c>
       <c r="B257" t="n">
-        <v>63486</v>
+        <v>255</v>
       </c>
       <c r="C257" t="n">
-        <v>65459</v>
+        <v>255</v>
       </c>
     </row>
   </sheetData>

</xml_diff>